<commit_message>
GRN | Handle optional Select Current Page dialog + config update
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/po-numbers.xlsx
+++ b/tests/po-numbers.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -35,6 +35,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -66,9 +72,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -382,7 +391,7 @@
   <dimension ref="A1:A10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="3" width="11.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="4" width="11.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -392,48 +401,42 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
-        <v>1010033271</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+        <v>1010033315</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
       <c r="A3" s="2">
-        <v>1010033270</v>
+        <v>1010033316</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
-        <v>1010033272</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+        <v>1010033317</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
       <c r="A5" s="2">
-        <v>1010033273</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+        <v>1010033318</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="2">
-        <v>1010033274</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+        <v>1010033319</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
       <c r="A7" s="2">
-        <v>1010033275</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
-      <c r="A8" s="2">
-        <v>1010033276</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
-      <c r="A9" s="2">
-        <v>1010033277</v>
-      </c>
+        <v>1010033320</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
+      <c r="A8" s="2"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
+      <c r="A9" s="3"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="1">
-        <v>1010033278</v>
-      </c>
+      <c r="A10" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
pl- fix | po duplicate fix
</commit_message>
<xml_diff>
--- a/tests/po-numbers.xlsx
+++ b/tests/po-numbers.xlsx
@@ -388,7 +388,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="4" width="11.576428571428572" customWidth="1" bestFit="1"/>
@@ -401,42 +401,103 @@
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
       <c r="A2" s="1">
-        <v>1010033315</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="2">
-        <v>1010033316</v>
+        <v>1010033706</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+      <c r="A3" s="1">
+        <v>1010033707</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1">
-        <v>1010033317</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
-      <c r="A5" s="2">
-        <v>1010033318</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
-      <c r="A6" s="2">
-        <v>1010033319</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
-      <c r="A7" s="2">
-        <v>1010033320</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
-      <c r="A8" s="2"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
-      <c r="A9" s="3"/>
+        <v>1010033709</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+      <c r="A5" s="1">
+        <v>1010033708</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+      <c r="A6" s="1">
+        <v>1010033710</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+      <c r="A7" s="1">
+        <v>1010033711</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+      <c r="A8" s="1">
+        <v>1010033713</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
+      <c r="A9" s="2">
+        <v>1010033712</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
-      <c r="A10" s="2"/>
+      <c r="A10" s="3">
+        <v>1010033715</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
+      <c r="A11" s="3">
+        <v>1010033714</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
+      <c r="A12" s="3">
+        <v>1010033716</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="19.5">
+      <c r="A13" s="3">
+        <v>1010033717</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
+      <c r="A14" s="3">
+        <v>1010033718</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="19.5">
+      <c r="A15" s="3">
+        <v>1010033720</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="19.5">
+      <c r="A16" s="3">
+        <v>1010033719</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="19.5">
+      <c r="A17" s="3">
+        <v>1010033721</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
+      <c r="A18" s="3">
+        <v>1010033722</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
+      <c r="A19" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
+      <c r="A20" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
+      <c r="A21" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
+      <c r="A22" s="3"/>
+    </row>
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
+      <c r="A23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>